<commit_message>
market mapping 2026-09-30: rapport corrige + methode piece jointe zip documentee
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ULEjcp2d45CaWN5d9CyRRR
</commit_message>
<xml_diff>
--- a/outputs/humanup_market_mapping_2026-09-30.xlsx
+++ b/outputs/humanup_market_mapping_2026-09-30.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -808,376 +808,383 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conséquence qualité : la **fraîcheur « 7 derniers jours » n'est pas confirmée** pour la majorité des annonces. Les dates non vérifiables sont notées `Date: NC` en clair dans la colonne `notes`, sans extrapolation. De même, l'effectif est `NC` pour la grande majorité des entreprises (non vérifiable sans Pappers) : le plafond des 2000 salariés a donc été appliqué par exclusion des employeurs connus </t>
+          <t xml:space="preserve">Conséquence qualité : la **fraîcheur « 7 derniers jours » n'est pas confirmée** pour la majorité des annonces. Attention à la lecture de la colonne `notes` : le champ `Date:` porte la date de mapping (2026-09-30) conformément au format d'import, **pas la date de publication de l'annonce**. L'incertitude sur la date de publication est signalée en clair dans le texte du champ `notes`, sur 100 % des </t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>## Top régions / villes / secteurs</t>
+          <t>De même, l'effectif est `NC` pour la grande majorité des entreprises (non vérifiable sans Pappers) : le plafond des 2000 salariés a donc été appliqué par exclusion des employeurs connus comme dépassant le seuil, pas par vérification systématique.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>**Départements** : Paris 75 (40 lignes), Loire-Atlantique 44 (11), Moselle 57 (8), Bouches-du-Rhône 13 (6), Haute-Garonne 31 (6), Côte-d'Or 21 (6), Gironde 33 (5), Corse-du-Sud 2A (4), Indre-et-Loire 37 (4), Isère 38 (4).</t>
+          <t>## Top régions / villes / secteurs</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>**Villes** : Paris (40), Aix-en-Provence, Tours, Toulouse, Reims, Cannes, Lyon, Bordeaux, Brest, Nantes (4 chacune), Ajaccio (2). 32 lignes en localisation `NC`.</t>
+          <t>**Départements** : Paris 75 (40 lignes), Loire-Atlantique 44 (11), Moselle 57 (8), Bouches-du-Rhône 13 (6), Haute-Garonne 31 (6), Côte-d'Or 21 (6), Gironde 33 (5), Corse-du-Sud 2A (4), Indre-et-Loire 37 (4), Isère 38 (4).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>**Secteurs dominants** : agroalimentaire et industrie de transformation, hôtellerie indépendante et châteaux-hôtels, cabinets d'expertise comptable régionaux, éditeurs SaaS B2B sous-médiatisés, distribution technique B2B (CVC, emballage).</t>
+          <t>**Villes** : Paris (40), Aix-en-Provence, Tours, Toulouse, Reims, Cannes, Lyon, Bordeaux, Brest, Nantes (4 chacune), Ajaccio (2). 32 lignes en localisation `NC`.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>**Équilibre géographique** : la consigne « privilégier les régions vs Paris/IdF » est respectée sur l'Industrie (Saint-Gérand 56, Torcheville 57, Vert-le-Grand 91) et le Sales général (Tours, Caen, La Roche-sur-Yon). La concentration parisienne vient surtout de Finance et Sales SaaS.</t>
+          <t>**Secteurs dominants** : agroalimentaire et industrie de transformation, hôtellerie indépendante et châteaux-hôtels, cabinets d'expertise comptable régionaux, éditeurs SaaS B2B sous-médiatisés, distribution technique B2B (CVC, emballage).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>## Top 7 signaux business prioritaires</t>
+          <t>**Équilibre géographique** : la consigne « privilégier les régions vs Paris/IdF » est respectée sur l'Industrie (Saint-Gérand 56, Torcheville 57, Vert-le-Grand 91) et le Sales général (Tours, Caen, La Roche-sur-Yon). La concentration parisienne vient surtout de Finance et Sales SaaS.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1. **Altho (marque Brets)** — Saint-Gérand (56) — 95 M€ investis dans une nouvelle usine, 443 salariés, CA 280 M€, DG Laurent Cavard nommé, montée en capacité à 25 000 t. Besoins production / maintenance / qualité massifs et durables. *→ Alexis*</t>
+          <t>## Top 7 signaux business prioritaires</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2. **Castellet Hospitality** — sortie du minoritaire Three Hills Capital Partners, capital majoritaire repris par le fondateur Gilles Larrivé et des family offices (Hospitality ON, sept. 2026). Recomposition capitalistique = fenêtre de recrutement. *→ Valentin*</t>
+          <t>1. **Altho (marque Brets)** — Saint-Gérand (56) — 95 M€ investis dans une nouvelle usine, 443 salariés, CA 280 M€, DG Laurent Cavard nommé, montée en capacité à 25 000 t. Besoins production / maintenance / qualité massifs et durables. *→ Alexis*</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>3. **Europa Group** — Toulouse (31) — 535 salariés, 160 M€ — LBO secondaire via fonds de continuation Abenex + build-up annoncé le 28/09/2026 (Life Science Access Academy, après K.I.T Group Berlin). Besoin conso / intercos / contrôle de gestion groupe. *→ Valentin*</t>
+          <t>2. **Castellet Hospitality** — sortie du minoritaire Three Hills Capital Partners, capital majoritaire repris par le fondateur Gilles Larrivé et des family offices (Hospitality ON, sept. 2026). Recomposition capitalistique = fenêtre de recrutement. *→ Valentin*</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>4. **Mistertemp' group** — ~1100 collaborateurs, intérim digital indépendant — création de la fonction Trésorerie &amp; Financements avec une équipe cible de 4-5 personnes (assurance-crédit, factor, reporting bancaire). Chantier de structuration complet, plusieurs postes à la clé. *→ Valentin*</t>
+          <t>3. **Europa Group** — Toulouse (31) — 535 salariés, 160 M€ — LBO secondaire via fonds de continuation Abenex + build-up annoncé le 28/09/2026 (Life Science Access Academy, après K.I.T Group Berlin). Besoin conso / intercos / contrôle de gestion groupe. *→ Valentin*</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>5. **Chapitre Six** — rachat de l'hôtel 3.14 à Cannes au Groupe Partouche (&gt;5 000 m²), plus grosse opération du groupe, réouverture 5* en 2027, plus projets Megève / Courchevel 1850 / Bus Palladium Paris. *→ Valentin*</t>
+          <t>4. **Mistertemp' group** — ~1100 collaborateurs, intérim digital indépendant — création de la fonction Trésorerie &amp; Financements avec une équipe cible de 4-5 personnes (assurance-crédit, factor, reporting bancaire). Chantier de structuration complet, plusieurs postes à la clé. *→ Valentin*</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>6. **ecosio** — recrute son **premier** Account Executive France, ouverture du marché français adossée au mandat e-invoicing de septembre 2026. Création d'une équipe commerciale from scratch. *→ Louis*</t>
+          <t>5. **Chapitre Six** — rachat de l'hôtel 3.14 à Cannes au Groupe Partouche (&gt;5 000 m²), plus grosse opération du groupe, réouverture 5* en 2027, plus projets Megève / Courchevel 1850 / Bus Palladium Paris. *→ Valentin*</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>7. **Le Comptoir CVC** — 3 annonces simultanées de technico-commerciaux itinérants (Tours 37, Caen 14, La Roche-sur-Yon 85) = extension de force de vente sur trois régions d'un coup. *→ Méroë*</t>
+          <t>6. **ecosio** — recrute son **premier** Account Executive France, ouverture du marché français adossée au mandat e-invoicing de septembre 2026. Création d'une équipe commerciale from scratch. *→ Louis*</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>**Signaux secondaires notables** : Axiome Associés (Christophe Delon élu président + intégration de 2 cabinets dans l'Hérault) ; Corse Composites Aéronautiques (Cadre Comptable en direct + 6 postes Qualité/Méthodes) ; SEMARDEL (4 postes maintenance ouverts simultanément) ; Loré (LBO primaire idiCo 8 M€ le 11/09/2026) ; GDCom Group (création d'un poste Grands Comptes Packaging, C1 et C2 nominatifs)</t>
+          <t>7. **Le Comptoir CVC** — 3 annonces simultanées de technico-commerciaux itinérants (Tours 37, Caen 14, La Roche-sur-Yon 85) = extension de force de vente sur trois régions d'un coup. *→ Méroë*</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>## Levées de fonds et opérations PE du jour (fichier de Louis)</t>
+          <t>**Signaux secondaires notables** : Axiome Associés (Christophe Delon élu président + intégration de 2 cabinets dans l'Hérault) ; Corse Composites Aéronautiques (Cadre Comptable en direct + 6 postes Qualité/Méthodes) ; SEMARDEL (4 postes maintenance ouverts simultanément) ; Loré (LBO primaire idiCo 8 M€ le 11/09/2026) ; GDCom Group (création d'un poste Grands Comptes Packaging, C1 et C2 nominatifs)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>| Société | Fonds | Montant | Nature | Date |</t>
+          <t>## Levées de fonds et opérations PE du jour (fichier de Louis)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>|---|---|---|---|---|</t>
+          <t>| Société | Fonds | Montant | Nature | Date |</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>| Loré (Bordeaux) | idiCo — fonds idiCo Expansion 4 | 8 M€ | LBO primaire + build-up Apoca | 11/09/2026 |</t>
+          <t>|---|---|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>| Kheops | Odyssée Venture + ISAI + Elaia | 12 M€ (15 M€ selon une autre source, à reconfirmer) | Levée | S39 2026 |</t>
+          <t>| Loré (Bordeaux) | idiCo — fonds idiCo Expansion 4 | 8 M€ | LBO primaire + build-up Apoca | 11/09/2026 |</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>| Zeliq | NC | 7 M€ | Levée | S39 2026 |</t>
+          <t>| Kheops | Odyssée Venture + ISAI + Elaia | 12 M€ (15 M€ selon une autre source, à reconfirmer) | Levée | S39 2026 |</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>| Beamy | NC | 8 M€ | Série A, déploiement international | Non confirmée |</t>
+          <t>| Zeliq | NC | 7 M€ | Levée | S39 2026 |</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>| EasyVista | NC | NC | Build-up | 2026, non confirmée |</t>
+          <t>| Beamy | NC | 8 M€ | Série A, déploiement international | Non confirmée |</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>## Récurrences</t>
+          <t>| EasyVista | NC | NC | Build-up | 2026, non confirmée |</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>**Aucune récurrence confirmée sur la fenêtre 23 → 30 septembre 2026.**</t>
+          <t>## Récurrences</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>31 des 214 entreprises déjà ciblées ces 14 derniers jours ont été re-testées. Aucun résultat de presse économique française postérieur au ~22 septembre n'est remonté : la semaine ne semble pas encore indexée, et tous les domaines permettant de vérifier une date sont bloqués par le proxy. Rien n'a été retenu plutôt que de forcer des dates incertaines. 16 entreprises restent non testées faute de bud</t>
+          <t>**Aucune récurrence confirmée sur la fenêtre 23 → 30 septembre 2026.**</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Trois signaux forts mais **hors fenêtre 7 jours** (18-22 septembre, datés et vérifiables), à traiter comme du rattrapage :</t>
+          <t>31 des 214 entreprises déjà ciblées ces 14 derniers jours ont été re-testées. Aucun résultat de presse économique française postérieur au ~22 septembre n'est remonté : la semaine ne semble pas encore indexée, et tous les domaines permettant de vérifier une date sont bloqués par le proxy. Rien n'a été retenu plutôt que de forcer des dates incertaines. 16 entreprises restent non testées faute de bud</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>- **PAREF Gestion** (Paris) — 3 nominations commerciales d'un coup (directeur réseaux de distribution + 2 responsables partenariats), 18/09 → structuration commerciale.</t>
+          <t>Trois signaux forts mais **hors fenêtre 7 jours** (18-22 septembre, datés et vérifiables), à traiter comme du rattrapage :</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>- **Stoïk** (Paris) — Xavier Marguinaud nommé VP Insurance, objectif &gt; 210 salariés fin 2026 après une série C de 20 M€, 18/09.</t>
+          <t>- **PAREF Gestion** (Paris) — 3 nominations commerciales d'un coup (directeur réseaux de distribution + 2 responsables partenariats), 18/09 → structuration commerciale.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>- **BIO-UV Group** (Lunel) — 4 responsables commerciaux recrutés + 2 promotions sur la force de vente Piscine, ~22/09.</t>
+          <t>- **Stoïk** (Paris) — Xavier Marguinaud nommé VP Insurance, objectif &gt; 210 salariés fin 2026 après une série C de 20 M€, 18/09.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>## 🔴 Alertes pipeline — entreprises à sortir du ciblage</t>
+          <t>- **BIO-UV Group** (Lunel) — 4 responsables commerciaux recrutés + 2 promotions sur la force de vente Piscine, ~22/09.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>- **Tessan** — en redressement judiciaire depuis le 28/04/2026.</t>
+          <t>## 🔴 Alertes pipeline — entreprises à sortir du ciblage</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>- **Groupe Okwind** — sous PSE, ~89 postes menacés.</t>
+          <t>- **Tessan** — en redressement judiciaire depuis le 28/04/2026.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>## Filtres appliqués</t>
+          <t>- **Groupe Okwind** — sous PSE, ~89 postes menacés.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>**Anti-doublons** : 214 entreprises ciblées sur les 14 derniers jours (32 fichiers scannés) ont été exclues de la recherche. Zéro collision constatée dans les 5 fichiers livrés.</t>
+          <t>## Filtres appliqués</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>**Plafond 2000 salariés (niveau groupe)** — exclusions explicites relevées par les agents : Réside Études, Korian, Cooperl, E.Leclerc, EDF/Framatome, SETEC, Paris Habitat, Descours &amp; Cabaud, Rydge Tie-up, Maïsadour, Septeo, Funecap, Givenchy/LVMH, Caisse d'Épargne IDF, Starbucks France, Rexel, Wilo, Lallemand, Chausson Matériaux, Petit Navire/Thai Union, Groupe Bodemer, Bouygues Telecom, d'aucy, V</t>
+          <t>**Anti-doublons** : 214 entreprises ciblées sur les 14 derniers jours (32 fichiers scannés) ont été exclues de la recherche. Zéro collision constatée dans les 5 fichiers livrés.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>**Liste noire** : aucune entreprise des Big 4, du next tier (Mazars, Grant Thornton, BDO, RSM, Baker Tilly), des réseaux d'expertise comptable (In Extenso, Fiducial, Cerfrance, Exco, Sofarec), des scale-ups trop visibles ni du CAC 40. Brevo, Libeo et Malt ont été écartés par l'agent Sales SaaS pour surexposition médiatique.</t>
+          <t>**Plafond 2000 salariés (niveau groupe)** — exclusions explicites relevées par les agents : Réside Études, Korian, Cooperl, E.Leclerc, EDF/Framatome, SETEC, Paris Habitat, Descours &amp; Cabaud, Rydge Tie-up, Maïsadour, Septeo, Funecap, Givenchy/LVMH, Caisse d'Épargne IDF, Starbucks France, Rexel, Wilo, Lallemand, Chausson Matériaux, Petit Navire/Thai Union, Groupe Bodemer, Bouygues Telecom, d'aucy, V</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>**Chaînes hôtelières** : aucun établissement Accor, Marriott, Hilton, IHG, Hyatt, Rosewood, Four Seasons ou Mandarin Oriental. Les 20 opportunités Hospitality sont des hôtels indépendants, châteaux-hôtels, Relais &amp; Châteaux, resorts et holdings de restauration.</t>
+          <t>**Liste noire** : aucune entreprise des Big 4, du next tier (Mazars, Grant Thornton, BDO, RSM, Baker Tilly), des réseaux d'expertise comptable (In Extenso, Fiducial, Cerfrance, Exco, Sofarec), des scale-ups trop visibles ni du CAC 40. Brevo, Libeo et Malt ont été écartés par l'agent Sales SaaS pour surexposition médiatique.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Employeur masqué** : annonces écartées chez Michael Page, Fed Finance, Robert Half, Manpower, Randstad, Menway, Winsearch, Camo Groupe, Actual, Achil, Talenteeds, Tamarin, Zanaka, Jobglober, Tylia, Crit, Lynx RH.</t>
+          <t>**Chaînes hôtelières** : aucun établissement Accor, Marriott, Hilton, IHG, Hyatt, Rosewood, Four Seasons ou Mandarin Oriental. Les 20 opportunités Hospitality sont des hôtels indépendants, châteaux-hôtels, Relais &amp; Châteaux, resorts et holdings de restauration.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>**Alternance / stage** : aucune annonce retenue (AB Compta écartée pour mention « apprenti »).</t>
+          <t>**Employeur masqué** : annonces écartées chez Michael Page, Fed Finance, Robert Half, Manpower, Randstad, Menway, Winsearch, Camo Groupe, Actual, Achil, Talenteeds, Tamarin, Zanaka, Jobglober, Tylia, Crit, Lynx RH.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>**Effectif &lt; 5 salariés** : Kepplair Evolution, Greens du Monde et Cabinet JCM écartés par prudence, effectif non vérifiable.</t>
+          <t>**Alternance / stage** : aucune annonce retenue (AB Compta écartée pour mention « apprenti »).</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Titres hors périmètre Industrie** : aucun Business Developer, Head of, VP ou Chief dans le fichier d'Alexis.</t>
+          <t>**Effectif &lt; 5 salariés** : Kepplair Evolution, Greens du Monde et Cabinet JCM écartés par prudence, effectif non vérifiable.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>## Dédoublonnage Sales Louis ↔ Méroë</t>
+          <t>**Titres hors périmètre Industrie** : aucun Business Developer, Head of, VP ou Chief dans le fichier d'Alexis.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>**Aucune entreprise retirée.** Les 14 entreprises du fichier de Louis et les 20 du fichier de Méroë sont disjointes — la consigne de séparation sectorielle (SaaS pur chez Louis, secteurs non-SaaS chez Méroë) a bien fonctionné en amont. Le fichier de Méroë est livré complet à 40 lignes.</t>
+          <t>## Dédoublonnage Sales Louis ↔ Méroë</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>## Volumes non atteints — best-effort assumé</t>
+          <t>**Aucune entreprise retirée.** Les 14 entreprises du fichier de Louis et les 20 du fichier de Méroë sont disjointes — la consigne de séparation sectorielle (SaaS pur chez Louis, secteurs non-SaaS chez Méroë) a bien fonctionné en amont. Le fichier de Méroë est livré complet à 40 lignes.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>- **Sales SaaS (Louis)** : 14 opportunités sur 20, 28 lignes sur 40. Budget de recherche épuisé après ~12 requêtes, et tous les domaines de la presse tech française bloqués par le proxy.</t>
+          <t>## Volumes non atteints — best-effort assumé</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>- **Sales général (Méroë)** : 17 JOB + 3 NEWS au lieu de 14 + 6. Le volume total de 40 lignes est atteint, mais la part NEWS est faible : BIO-UV était déjà dans l'anti-doublons, et d'aucy / Volvo / Seat / NGE / SEB dépassaient le plafond groupe.</t>
+          <t>- **Sales SaaS (Louis)** : 14 opportunités sur 20, 28 lignes sur 40. Budget de recherche épuisé après ~12 requêtes, et tous les domaines de la presse tech française bloqués par le proxy.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>- **Industrie** : les familles logistique industrielle, chantier, technico-commercial industriel, achats et direction de site n'ont pas été couvertes, budget de recherche épuisé avant.</t>
+          <t>- **Sales général (Méroë)** : 17 JOB + 3 NEWS au lieu de 14 + 6. Le volume total de 40 lignes est atteint, mais la part NEWS est faible : BIO-UV était déjà dans l'anti-doublons, et d'aucy / Volvo / Seat / NGE / SEB dépassaient le plafond groupe.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>## Actions recommandées</t>
+          <t>- **Industrie** : les familles logistique industrielle, chantier, technico-commercial industriel, achats et direction de site n'ont pas été couvertes, budget de recherche épuisé avant.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>1. **Enrichir avant d'appeler** : lancer FullEnrich à l'import Propium sur les 169 lignes `CONTACT_NON_SOURCE`, en commençant par les 7 signaux prioritaires ci-dessus.</t>
+          <t>## Actions recommandées</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2. **Revalider les dates** : la fraîcheur 7 jours n'est pas garantie. Vérifier la date de publication avant d'attaquer une annonce, surtout sur Finance A/B/C et Hospitality.</t>
+          <t>1. **Enrichir avant d'appeler** : lancer FullEnrich à l'import Propium sur les 169 lignes `CONTACT_NON_SOURCE`, en commençant par les 7 signaux prioritaires ci-dessus.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>3. **Sortir Tessan et Groupe Okwind** du pipe.</t>
+          <t>2. **Revalider les dates** : la fraîcheur 7 jours n'est pas garantie. Le champ `Date:` des notes est la date de mapping, pas celle de l'annonce — vérifier la date de publication via le lien avant d'attaquer, surtout sur Finance et Hospitality.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>4. **Rattraper les 3 signaux hors fenêtre** (PAREF Gestion, Stoïk, BIO-UV Group) : ils sont datés et vérifiables.</t>
+          <t>3. **Sortir Tessan et Groupe Okwind** du pipe.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
+        <is>
+          <t>4. **Rattraper les 3 signaux hors fenêtre** (PAREF Gestion, Stoïk, BIO-UV Group) : ils sont datés et vérifiables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
         <is>
           <t>5. **Relancer une passe de récurrences dans 3-4 jours** sur les 16 entreprises non testées.</t>
         </is>

</xml_diff>

<commit_message>
market mapping 2026-09-30: incident de livraison louis@humanup.io (550 5.7.1)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ULEjcp2d45CaWN5d9CyRRR
</commit_message>
<xml_diff>
--- a/outputs/humanup_market_mapping_2026-09-30.xlsx
+++ b/outputs/humanup_market_mapping_2026-09-30.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1151,42 +1151,175 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>## Actions recommandées</t>
+          <t>## 🔴 Incident de livraison — la boîte de Louis rejette tous les emails</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>1. **Enrichir avant d'appeler** : lancer FullEnrich à l'import Propium sur les 169 lignes `CONTACT_NON_SOURCE`, en commençant par les 7 signaux prioritaires ci-dessus.</t>
+          <t>L'email du jour destiné à `louis@humanup.io` a été **rejeté par le serveur** :</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2. **Revalider les dates** : la fraîcheur 7 jours n'est pas garantie. Le champ `Date:` des notes est la date de mapping, pas celle de l'annonce — vérifier la date de publication via le lien avant d'attaquer, surtout sur Finance et Hospitality.</t>
+          <t>```</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>3. **Sortir Tessan et Groupe Okwind** du pipe.</t>
+          <t>550 5.7.1 Your message was not delivered because the recipient is unable to</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>4. **Rattraper les 3 signaux hors fenêtre** (PAREF Gestion, Stoïk, BIO-UV Group) : ils sont datés et vérifiables.</t>
+          <t>receive email. You can contact meroe@humanup.io instead.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
+          <t>```</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Ce n'est ni un problème de pièce jointe ni de format : la boîte est hors service au niveau de l'administration Google Workspace, et le rebond redirige explicitement vers `meroe@humanup.io`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>**Ce n'est pas nouveau** : le même rejet s'est produit le 29/09 à 06:54 et à 08:27, sur des envois sans archive ZIP. Louis n'a donc reçu aucun fichier depuis au moins deux jours, et les runs précédents ne l'ont pas détecté — aucun n'avait vérifié les rebonds après envoi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Décision à prendre : soit réactiver la boîte dans la console Google Workspace (ou corriger la règle de routage), soit retirer Louis de la liste de diffusion comme cela a été fait pour Marie Le Ret, pour éviter un rebond quotidien.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>En attendant, `sales_saas_2026-09-30.csv` a été renvoyé à Méroë.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>## Statut d'envoi des 4 emails</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>| Destinataire | Fichiers | Statut |</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>|---|---|---|</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>| valentin@humanup.io | finance + hospitality (ZIP) | ✅ Délivré |</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>| alexis@humanup.io | industrie (ZIP) | ✅ Délivré |</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>| louis@humanup.io | sales_saas (ZIP) | ❌ **Rejeté 550 5.7.1** — rerouté vers Méroë |</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>| meroe@humanup.io | sales (ZIP) + rapport en corps | ✅ Délivré |</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>**Note technique sur les pièces jointes** : les CSV partent désormais en archive ZIP (à dézipper avant l'import Propium). Le connecteur Gmail exige un base64 inline dans l'appel d'outil ; un CSV brut de 26 Ko représente ~53 000 tokens de sortie, au-delà de ce qu'un appel peut porter — c'est ce qui avait fait partir un CSV tronqué lors d'un run précédent. Zippé, le payload tombe sous 8 000 caractèr</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>## Actions recommandées</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>1. **Enrichir avant d'appeler** : lancer FullEnrich à l'import Propium sur les 169 lignes `CONTACT_NON_SOURCE`, en commençant par les 7 signaux prioritaires ci-dessus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2. **Revalider les dates** : la fraîcheur 7 jours n'est pas garantie. Le champ `Date:` des notes est la date de mapping, pas celle de l'annonce — vérifier la date de publication via le lien avant d'attaquer, surtout sur Finance et Hospitality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>3. **Sortir Tessan et Groupe Okwind** du pipe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>4. **Rattraper les 3 signaux hors fenêtre** (PAREF Gestion, Stoïk, BIO-UV Group) : ils sont datés et vérifiables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
           <t>5. **Relancer une passe de récurrences dans 3-4 jours** sur les 16 entreprises non testées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>6. **Trancher le cas de la boîte de Louis** (réactivation ou retrait de la diffusion) — c'est la seule action bloquante pour le run de demain.</t>
         </is>
       </c>
     </row>

</xml_diff>